<commit_message>
Diagrama blocs versió 4 + BOM actualitzat + Bus CAN i USART + Lector RFID
</commit_message>
<xml_diff>
--- a/BOM_Projecte_Eines_Disseny.xlsx
+++ b/BOM_Projecte_Eines_Disseny.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="41">
   <si>
     <t>Component</t>
   </si>
@@ -73,19 +73,40 @@
     <t>511-VNH5019A-E</t>
   </si>
   <si>
+    <t xml:space="preserve">ACI 83094 </t>
+  </si>
+  <si>
     <t>Motor alçavidres</t>
   </si>
   <si>
+    <t>AutoZone</t>
+  </si>
+  <si>
+    <t>2x</t>
+  </si>
+  <si>
+    <t>CINCHING LATCH MOTOR</t>
+  </si>
+  <si>
     <t>Motor actuador porta</t>
   </si>
   <si>
-    <t>MFDRC522</t>
+    <t>Johnson Electronics</t>
+  </si>
+  <si>
+    <t>2X</t>
+  </si>
+  <si>
+    <t>RC522</t>
   </si>
   <si>
     <t>Lector RFID</t>
   </si>
   <si>
-    <t>771-MFRC52201HN1157</t>
+    <t>Modulo RFID RC522</t>
+  </si>
+  <si>
+    <t>ElectroComponentes</t>
   </si>
   <si>
     <t>SN65HVD230</t>
@@ -104,6 +125,15 @@
   </si>
   <si>
     <t>653-SS-5GLD</t>
+  </si>
+  <si>
+    <t>LM2596S-5.0</t>
+  </si>
+  <si>
+    <t>DC-DC</t>
+  </si>
+  <si>
+    <t>926-LM2596S-ADJ/NOPB</t>
   </si>
 </sst>
 </file>
@@ -134,6 +164,7 @@
     <font>
       <u/>
       <color rgb="FF0000FF"/>
+      <name val="Roboto"/>
     </font>
   </fonts>
   <fills count="2">
@@ -144,37 +175,35 @@
       <patternFill patternType="lightGray"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border/>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
@@ -191,7 +220,69 @@
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="5">
+    <dxf>
+      <font/>
+      <fill>
+        <patternFill patternType="none"/>
+      </fill>
+      <border/>
+    </dxf>
+    <dxf>
+      <font/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF356854"/>
+          <bgColor rgb="FF356854"/>
+        </patternFill>
+      </fill>
+      <border/>
+    </dxf>
+    <dxf>
+      <font/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <border/>
+    </dxf>
+    <dxf>
+      <font/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+      <border/>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF356854"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF356854"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF356854"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF356854"/>
+        </bottom>
+      </border>
+    </dxf>
+  </dxfs>
+  <tableStyles count="1">
+    <tableStyle count="4" pivot="0" name="BOM-style">
+      <tableStyleElement dxfId="1" type="headerRow"/>
+      <tableStyleElement dxfId="2" type="firstRowStripe"/>
+      <tableStyleElement dxfId="3" type="secondRowStripe"/>
+      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    </tableStyle>
+  </tableStyles>
 </styleSheet>
 </file>
 
@@ -201,6 +292,22 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A2:H11" displayName="Tabla_1" name="Tabla_1" id="1">
+  <tableColumns count="8">
+    <tableColumn name="Component" id="1"/>
+    <tableColumn name="Descripció" id="2"/>
+    <tableColumn name="Ref. Fabricant" id="3"/>
+    <tableColumn name="Package" id="4"/>
+    <tableColumn name="Datasheet" id="5"/>
+    <tableColumn name="Proveïdor" id="6"/>
+    <tableColumn name="Preu" id="7"/>
+    <tableColumn name="Unitats" id="8"/>
+  </tableColumns>
+  <tableStyleInfo name="BOM-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -404,12 +511,14 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="17.63"/>
-    <col customWidth="1" min="2" max="2" width="18.63"/>
+    <col customWidth="1" min="1" max="1" width="22.25"/>
+    <col customWidth="1" min="2" max="2" width="18.88"/>
     <col customWidth="1" min="3" max="3" width="22.13"/>
+    <col customWidth="1" min="5" max="5" width="13.13"/>
+    <col customWidth="1" min="6" max="6" width="17.38"/>
   </cols>
   <sheetData>
-    <row r="2">
+    <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -435,7 +544,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
@@ -459,7 +568,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>13</v>
       </c>
@@ -483,7 +592,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="22.5" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
@@ -507,63 +616,77 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="5"/>
+    <row r="6" ht="22.5" customHeight="1">
+      <c r="A6" s="2" t="s">
+        <v>20</v>
+      </c>
       <c r="B6" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="5"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="5"/>
+      <c r="F6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G6" s="4">
+        <v>74.99</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" ht="22.5" customHeight="1">
+      <c r="A7" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="B7" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="5"/>
-    </row>
-    <row r="8">
+      <c r="F7" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G7" s="4">
+        <v>30.0</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" ht="22.5" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="D8" s="5"/>
-      <c r="E8" s="3" t="s">
-        <v>4</v>
-      </c>
+      <c r="E8" s="6"/>
       <c r="F8" s="3" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="G8" s="4">
-        <v>6.41</v>
+        <v>2.2</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="3" t="s">
@@ -579,15 +702,15 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="22.5" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="3" t="s">
@@ -603,120 +726,139 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="5"/>
+    <row r="11" ht="22.5" customHeight="1">
+      <c r="A11" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" s="2"/>
+      <c r="E11" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G11" s="4">
+        <v>5.99</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="5"/>
+      <c r="A12" s="7"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="7"/>
     </row>
     <row r="13">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="5"/>
+      <c r="A13" s="7"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="7"/>
     </row>
     <row r="14">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="5"/>
+      <c r="A14" s="7"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="7"/>
     </row>
     <row r="15">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="5"/>
+      <c r="A15" s="7"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="7"/>
     </row>
     <row r="16">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="5"/>
+      <c r="A16" s="7"/>
+      <c r="B16" s="7"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="7"/>
     </row>
     <row r="17">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="5"/>
+      <c r="A17" s="9"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="9"/>
     </row>
     <row r="18">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="5"/>
+      <c r="A18" s="9"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="9"/>
     </row>
     <row r="19">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="6"/>
-      <c r="H19" s="5"/>
+      <c r="A19" s="9"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="9"/>
     </row>
     <row r="20">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="6"/>
-      <c r="H20" s="5"/>
+      <c r="A20" s="9"/>
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="9"/>
     </row>
     <row r="21">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="5"/>
+      <c r="A21" s="9"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="9"/>
     </row>
     <row r="22">
-      <c r="G22" s="7"/>
+      <c r="G22" s="11"/>
     </row>
   </sheetData>
+  <dataValidations>
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="G3:G11">
+      <formula1>AND(ISNUMBER(G3),(NOT(OR(NOT(ISERROR(DATEVALUE(G3))), AND(ISNUMBER(G3), LEFT(CELL("format", G3))="D")))))</formula1>
+    </dataValidation>
+  </dataValidations>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="E3"/>
     <hyperlink r:id="rId2" ref="F3"/>
@@ -724,13 +866,19 @@
     <hyperlink r:id="rId4" ref="F4"/>
     <hyperlink r:id="rId5" ref="E5"/>
     <hyperlink r:id="rId6" ref="F5"/>
-    <hyperlink r:id="rId7" ref="E8"/>
-    <hyperlink r:id="rId8" ref="F8"/>
-    <hyperlink r:id="rId9" ref="E9"/>
-    <hyperlink r:id="rId10" ref="F9"/>
-    <hyperlink r:id="rId11" ref="E10"/>
-    <hyperlink r:id="rId12" ref="F10"/>
+    <hyperlink r:id="rId7" ref="F6"/>
+    <hyperlink r:id="rId8" ref="F7"/>
+    <hyperlink r:id="rId9" ref="F8"/>
+    <hyperlink r:id="rId10" ref="E9"/>
+    <hyperlink r:id="rId11" ref="F9"/>
+    <hyperlink r:id="rId12" ref="E10"/>
+    <hyperlink r:id="rId13" ref="F10"/>
+    <hyperlink r:id="rId14" ref="E11"/>
+    <hyperlink r:id="rId15" ref="F11"/>
   </hyperlinks>
-  <drawing r:id="rId13"/>
+  <drawing r:id="rId16"/>
+  <tableParts count="1">
+    <tablePart r:id="rId18"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>